<commit_message>
feat: separate quick replies and open reply table from screen edges
</commit_message>
<xml_diff>
--- a/apps/web/static/script-template.xlsx
+++ b/apps/web/static/script-template.xlsx
@@ -33,35 +33,40 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t xml:space="preserve">kind</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t xml:space="preserve">isEntry</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t xml:space="preserve">reply:zh-CN</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t xml:space="preserve">reply:ko</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t xml:space="preserve">reply:en</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t xml:space="preserve">variables</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t xml:space="preserve">branches</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t xml:space="preserve">materialIds</t>
         </is>
@@ -90,35 +95,40 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t xml:space="preserve">flow</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t xml:space="preserve">true</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t xml:space="preserve">您好，{客户姓名}，吃饭了吗？</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t xml:space="preserve">{客户姓名}님, 식사하셨어요?</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t xml:space="preserve">Hello {客户姓名}, have you eaten?</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t xml:space="preserve">[{"name": "客户姓名", "label": "客户姓名", "required": true}]</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t xml:space="preserve">[{"id": "start-yes", "label": "吃了", "targetId": "yes"}, {"id": "start-no", "label": "还没吃", "targetId": "no"}]</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t xml:space="preserve">[]</t>
         </is>
@@ -147,35 +157,40 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t xml:space="preserve">flow</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t xml:space="preserve">false</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t xml:space="preserve">祝您今天愉快！</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t xml:space="preserve">좋은 하루 보내세요!</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t xml:space="preserve">Have a lovely day!</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[]</t>
-        </is>
-      </c>
       <c r="J3" t="inlineStr">
         <is>
+          <t xml:space="preserve">[]</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
           <t xml:space="preserve">[{"id":"yes-next","label":"继续","targetId":"product"}]</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t xml:space="preserve">[]</t>
         </is>
@@ -204,35 +219,40 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t xml:space="preserve">flow</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t xml:space="preserve">false</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t xml:space="preserve">记得按时吃饭。</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t xml:space="preserve">식사 꼭 챙기세요.</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t xml:space="preserve">Remember to eat on time.</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[]</t>
-        </is>
-      </c>
       <c r="J4" t="inlineStr">
         <is>
+          <t xml:space="preserve">[]</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
           <t xml:space="preserve">[{"id":"no-next","label":"继续","targetId":"product"}]</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t xml:space="preserve">[]</t>
         </is>
@@ -261,35 +281,40 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t xml:space="preserve">flow</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t xml:space="preserve">false</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t xml:space="preserve">我把详细资料发给您。</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t xml:space="preserve">자세한 자료를 보내드릴게요.</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t xml:space="preserve">I will send you the details.</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">[]</t>
-        </is>
-      </c>
       <c r="J5" t="inlineStr">
         <is>
           <t xml:space="preserve">[]</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[]</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t xml:space="preserve">[]</t>
         </is>

</xml_diff>